<commit_message>
Updated the English version of the data analysis script.
</commit_message>
<xml_diff>
--- a/original_data/data_source.xlsx
+++ b/original_data/data_source.xlsx
@@ -5,27 +5,38 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CASA\homelessness_research\original_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveuclac-my.sharepoint.com/personal/uceshc0_ucl_ac_uk/Documents/CASA/2025/dissertation/Dissertation_Yifan_Feng/homelessness_research/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C5C105E-0485-4273-AB8A-2E54592B3311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{0C5C105E-0485-4273-AB8A-2E54592B3311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E815AAAC-95B2-4D52-8046-40FFFE87A8A8}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>data</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -278,10 +289,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>population</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>MYE4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -303,6 +310,14 @@
   </si>
   <si>
     <t>page</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OpenStreetMap data, 2025</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Population</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -408,7 +423,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -425,13 +440,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -740,8 +749,8 @@
       <c r="E1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>48</v>
+      <c r="F1" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="96.9" customHeight="1" x14ac:dyDescent="0.35">
@@ -757,7 +766,7 @@
       <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -863,8 +872,8 @@
       <c r="D7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="3">
-        <v>2025</v>
+      <c r="E7" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="F7" s="3"/>
     </row>
@@ -881,33 +890,33 @@
       <c r="D8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="3">
-        <v>2025</v>
+      <c r="E8" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:7" ht="38.6" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="C10" s="7"/>
+      <c r="C10" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -921,5 +930,6 @@
     <hyperlink ref="D9" r:id="rId7" xr:uid="{3914A45C-6556-4092-A14E-DE229B1AB3FC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>